<commit_message>
TRIN 5.9.3 - Bernardo v2.4 homologado - Modulos 17 e 19 concluídos
</commit_message>
<xml_diff>
--- a/MARCO_ZERO_INSTITUCIONAL.xlsx
+++ b/MARCO_ZERO_INSTITUCIONAL.xlsx
@@ -156,96 +156,96 @@
 <volTypes xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <volType type="realTimeData">
     <main first="rtdtrading.rtdserver">
-      <tp t="e">
-        <v>#N/A</v>
+      <tp>
+        <v>169970</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>ABE</stp>
+        <tr r="E2" s="1"/>
         <tr r="W2" s="1"/>
-        <tr r="E2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      </tp>
+      <tp t="s">
+        <v>09/06/2026</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>DAT</stp>
         <tr r="T2" s="1"/>
         <tr r="B2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>18:31:28</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>HOR</stp>
         <tr r="U2" s="1"/>
         <tr r="C2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp>
+        <v>171205</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>MAX</stp>
+        <tr r="F2" s="1"/>
         <tr r="X2" s="1"/>
-        <tr r="F2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      </tp>
+      <tp>
+        <v>168710</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>MIN</stp>
         <tr r="Y2" s="1"/>
         <tr r="G2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp>
+        <v>170025</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>ULT</stp>
         <tr r="D2" s="1"/>
         <tr r="V2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp>
+        <v>723451389850</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>VOL</stp>
         <tr r="Z2" s="1"/>
         <tr r="H2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>-31.399,00</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>103</stp>
+        <tr r="J2" s="1"/>
         <tr r="AB2" s="1"/>
-        <tr r="J2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      </tp>
+      <tp t="s">
+        <v>-31.399</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>100</stp>
         <tr r="AD2" s="1"/>
         <tr r="L2" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>170.131</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>67</stp>
+        <tr r="N2" s="1"/>
         <tr r="AF2" s="1"/>
-        <tr r="N2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      </tp>
+      <tp t="s">
+        <v>8.004.510</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>98</stp>
+        <tr r="AC2" s="1"/>
         <tr r="K2" s="1"/>
-        <tr r="AC2" s="1"/>
-      </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      </tp>
+      <tp t="s">
+        <v>8.035.909</v>
         <stp/>
         <stp>WINM26_F_0</stp>
         <stp>99</stp>
@@ -635,114 +635,114 @@
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="e">
+      <c r="B2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "DAT")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="C2" s="2" t="e">
+        <v>09/06/2026</v>
+      </c>
+      <c r="C2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "HOR")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D2" s="2" t="e">
+        <v>18:31:28</v>
+      </c>
+      <c r="D2" s="2">
         <f>RTD("rtdtrading.rtdserver",,"WINM26_F_0","ULT")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E2" s="2" t="e">
+        <v>170025</v>
+      </c>
+      <c r="E2" s="2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "ABE")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F2" s="2" t="e">
+        <v>169970</v>
+      </c>
+      <c r="F2" s="2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "MAX")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G2" s="2" t="e">
+        <v>171205</v>
+      </c>
+      <c r="G2" s="2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "MIN")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H2" s="2" t="e">
+        <v>168710</v>
+      </c>
+      <c r="H2" s="2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "VOL")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="I2" s="3" t="e">
+        <v>723451389850</v>
+      </c>
+      <c r="I2" s="3" t="str">
         <f>L2</f>
-        <v>#N/A</v>
-      </c>
-      <c r="J2" s="2" t="e">
+        <v>-31.399</v>
+      </c>
+      <c r="J2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "103")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="K2" s="2" t="e">
+        <v>-31.399,00</v>
+      </c>
+      <c r="K2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "98")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="L2" s="2" t="e">
+        <v>8.004.510</v>
+      </c>
+      <c r="L2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "100")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="M2" s="2" t="e">
+        <v>-31.399</v>
+      </c>
+      <c r="M2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "99")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="N2" s="2" t="e">
+        <v>8.035.909</v>
+      </c>
+      <c r="N2" s="2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "67")</f>
-        <v>#N/A</v>
+        <v>170.131</v>
       </c>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
       <c r="S2" t="s">
         <v>13</v>
       </c>
-      <c r="T2" t="e">
+      <c r="T2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "DAT")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="U2" t="e">
+        <v>09/06/2026</v>
+      </c>
+      <c r="U2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "HOR")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="V2" t="e">
+        <v>18:31:28</v>
+      </c>
+      <c r="V2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "ULT")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="W2" t="e">
+        <v>170025</v>
+      </c>
+      <c r="W2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "ABE")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="X2" t="e">
+        <v>169970</v>
+      </c>
+      <c r="X2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "MAX")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Y2" t="e">
+        <v>171205</v>
+      </c>
+      <c r="Y2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "MIN")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="Z2" t="e">
+        <v>168710</v>
+      </c>
+      <c r="Z2">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "VOL")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AA2" s="3" t="e">
+        <v>723451389850</v>
+      </c>
+      <c r="AA2" s="3" t="str">
         <f>AD2</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AB2" t="e">
+        <v>-31.399</v>
+      </c>
+      <c r="AB2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "103")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AC2" t="e">
+        <v>-31.399,00</v>
+      </c>
+      <c r="AC2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "98")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AD2" t="e">
+        <v>8.004.510</v>
+      </c>
+      <c r="AD2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "100")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AE2" t="e">
+        <v>-31.399</v>
+      </c>
+      <c r="AE2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "99")</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AF2" t="e">
+        <v>8.035.909</v>
+      </c>
+      <c r="AF2" t="str">
         <f>RTD("rtdtrading.rtdserver",, "WINM26_F_0", "67")</f>
-        <v>#N/A</v>
+        <v>170.131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>